<commit_message>
Updated for EA 23.352 Patch 1 Stable. Added “Enable Context Menu” (enabled by default) to show or hide the free upgrade menu. Please review the new setting in Mod Config or the BepInEx config file after updating. EA 23.352 Patch 1 Stable に対応しました。無料の強化メニューの表示・非表示を切り替える「Enable Context Menu」（初期設定：オン）を追加しました。更新後は、Mod Config または BepInEx の設定ファイルで新しい設定をご確認ください。 已更新至 EA 23.352 Patch 1 Stable。新增“Enable Context Menu”设置（默认开启），可显示或隐藏免费升级菜单。更新后，请在 Mod Config 或 BepInEx 配置文件中查看此新设置。
</commit_message>
<xml_diff>
--- a/package/LangMod/EN/SourceContainerUpgrades.xlsx
+++ b/package/LangMod/EN/SourceContainerUpgrades.xlsx
@@ -1,29 +1,29 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="Calc"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
-  <workbookProtection/>
+  <workbookPr autoCompressPictures="1"/>
+  <workbookProtection lockStructure="0" lockWindows="0" lockRevision="0"/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView windowWidth="16384" windowHeight="8192" tabRatio="500"/>
   </bookViews>
   <sheets>
-    <sheet name="General" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="General" sheetId="1" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">General!$A$3:$D$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1"><![CDATA[General!$A$3:$D$4]]></definedName>
   </definedNames>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
+  <calcPr calcMode="auto" fullCalcOnLoad="0" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001" fullPrecision="1" calcCompleted="0" calcOnSave="0" concurrentCalc="0" forceFullCalc="0"/>
   <extLst>
-    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
+    <ext uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
+      <loext:extCalcPr xmlns:loext="http://schemas.libreoffice.org/" stringRefSyntax="ExcelA1"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="120">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="162" uniqueCount="122">
   <si>
     <t xml:space="preserve">id</t>
   </si>
@@ -383,6 +383,12 @@
   </si>
   <si>
     <t xml:space="preserve">Reduces the storage chest's max item capacity without changing its page grid size, if the current items still fit.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">コンテナ強化</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Container Upgrades</t>
   </si>
 </sst>
 </file>
@@ -403,17 +409,17 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
-      <family val="0"/>
+      <family/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
-      <family val="0"/>
+      <family/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
-      <family val="0"/>
+      <family/>
     </font>
     <font>
       <sz val="10"/>
@@ -458,14 +464,14 @@
     </fill>
   </fills>
   <borders count="2">
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left style="hair"/>
       <right style="hair"/>
       <top style="hair"/>
@@ -474,62 +480,62 @@
     </border>
   </borders>
   <cellStyleXfs count="21">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment/>
+      <protection locked="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="0"/>
+    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="0"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="0"/>
+    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="0"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="0"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment/>
+      <protection locked="1"/>
     </xf>
   </cellStyleXfs>
   <cellXfs count="7">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="0">
+      <alignment/>
+      <protection locked="1"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="20" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment/>
+      <protection locked="1"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="20" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="20" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment/>
+      <protection locked="1"/>
     </xf>
-    <xf numFmtId="165" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="165" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment/>
+      <protection locked="1"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="2" borderId="1" xfId="20" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="165" fontId="7" fillId="2" borderId="1" xfId="20" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment/>
+      <protection locked="1"/>
     </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment/>
+      <protection locked="1"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
+      <alignment/>
+      <protection locked="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="7">
@@ -539,7 +545,7 @@
     <cellStyle name="Currency" xfId="17" builtinId="4"/>
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
-    <cellStyle name="Excel Built-in Normal" xfId="20"/>
+    <cellStyle name="Excel Built-in Normal" xfId="20" builtinId="0"/>
   </cellStyles>
   <dxfs count="4">
     <dxf>
@@ -567,13 +573,13 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF9C0006"/>
         <name val="ヒラギノ角ゴ ProN W3"/>
+        <family val="2"/>
         <charset val="128"/>
-        <family val="2"/>
-        <color rgb="FF9C0006"/>
       </font>
       <fill>
-        <patternFill>
+        <patternFill patternType="solid">
           <bgColor rgb="FFFFC7CE"/>
         </patternFill>
       </fill>
@@ -643,7 +649,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -753,21 +759,21 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr>
+    <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I41"/>
-  <sheetFormatPr defaultColWidth="7.4296875" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="7.4296875" defaultRowHeight="12.8"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="23.84"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="17.87"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="59.91"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="51.2"/>
-    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="5" style="2" width="7.43"/>
+    <col min="1" max="1" width="23.84" style="1" customWidth="1"/>
+    <col min="2" max="2" width="17.87" style="1" customWidth="1"/>
+    <col min="3" max="3" width="59.91" style="1" customWidth="1"/>
+    <col min="4" max="4" width="51.2" style="1" customWidth="1"/>
+    <col min="5" max="16384" width="7.43" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" ht="13.8">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -781,7 +787,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" ht="13.8">
       <c r="A2" s="3" t="s">
         <v>4</v>
       </c>
@@ -795,13 +801,13 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" ht="13.8">
       <c r="A3" s="3"/>
       <c r="B3" s="3"/>
       <c r="C3" s="4"/>
       <c r="D3" s="4"/>
     </row>
-    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" ht="12.8">
       <c r="A4" s="5" t="s">
         <v>5</v>
       </c>
@@ -809,13 +815,13 @@
         <v>6</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>7</v>
+        <v>120</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5" s="6" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="5" s="6" customFormat="1" ht="12.8">
       <c r="A5" s="5" t="s">
         <v>9</v>
       </c>
@@ -834,7 +840,7 @@
       <c r="H5" s="2"/>
       <c r="I5" s="2"/>
     </row>
-    <row r="6" s="6" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" s="6" customFormat="1" ht="12.8">
       <c r="A6" s="5" t="s">
         <v>12</v>
       </c>
@@ -853,7 +859,7 @@
       <c r="H6" s="2"/>
       <c r="I6" s="2"/>
     </row>
-    <row r="7" s="6" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" s="6" customFormat="1" ht="12.8">
       <c r="A7" s="5" t="s">
         <v>15</v>
       </c>
@@ -872,7 +878,7 @@
       <c r="H7" s="2"/>
       <c r="I7" s="2"/>
     </row>
-    <row r="8" s="6" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" s="6" customFormat="1" ht="12.8">
       <c r="A8" s="5" t="s">
         <v>18</v>
       </c>
@@ -891,7 +897,7 @@
       <c r="H8" s="2"/>
       <c r="I8" s="2"/>
     </row>
-    <row r="9" s="6" customFormat="true" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" s="6" customFormat="1" ht="12.8">
       <c r="A9" s="5" t="s">
         <v>21</v>
       </c>
@@ -910,7 +916,7 @@
       <c r="H9" s="2"/>
       <c r="I9" s="2"/>
     </row>
-    <row r="10" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" ht="12.8">
       <c r="A10" s="5" t="s">
         <v>24</v>
       </c>
@@ -924,7 +930,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" ht="12.8">
       <c r="A11" s="5" t="s">
         <v>27</v>
       </c>
@@ -938,7 +944,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" ht="12.8">
       <c r="A12" s="5" t="s">
         <v>30</v>
       </c>
@@ -952,7 +958,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" ht="12.8">
       <c r="A13" s="5" t="s">
         <v>33</v>
       </c>
@@ -966,7 +972,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" ht="12.8">
       <c r="A14" s="5" t="s">
         <v>36</v>
       </c>
@@ -980,7 +986,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" ht="12.8">
       <c r="A15" s="5" t="s">
         <v>39</v>
       </c>
@@ -994,7 +1000,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" ht="12.8">
       <c r="A16" s="5" t="s">
         <v>42</v>
       </c>
@@ -1008,7 +1014,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" ht="12.8">
       <c r="A17" s="5" t="s">
         <v>45</v>
       </c>
@@ -1022,7 +1028,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" ht="12.8">
       <c r="A18" s="5" t="s">
         <v>48</v>
       </c>
@@ -1036,7 +1042,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" ht="12.8">
       <c r="A19" s="5" t="s">
         <v>51</v>
       </c>
@@ -1050,7 +1056,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" ht="12.8">
       <c r="A20" s="5" t="s">
         <v>54</v>
       </c>
@@ -1064,7 +1070,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" ht="12.8">
       <c r="A21" s="5" t="s">
         <v>57</v>
       </c>
@@ -1078,7 +1084,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" ht="12.8">
       <c r="A22" s="5" t="s">
         <v>60</v>
       </c>
@@ -1092,7 +1098,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" ht="12.8">
       <c r="A23" s="5" t="s">
         <v>63</v>
       </c>
@@ -1106,7 +1112,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" ht="12.8">
       <c r="A24" s="5" t="s">
         <v>66</v>
       </c>
@@ -1120,7 +1126,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" ht="12.8">
       <c r="A25" s="5" t="s">
         <v>69</v>
       </c>
@@ -1134,7 +1140,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="26" ht="12.8">
       <c r="A26" s="5" t="s">
         <v>72</v>
       </c>
@@ -1148,7 +1154,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="27" ht="12.8">
       <c r="A27" s="5" t="s">
         <v>75</v>
       </c>
@@ -1162,7 +1168,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="28" ht="12.8">
       <c r="A28" s="5" t="s">
         <v>78</v>
       </c>
@@ -1176,7 +1182,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="29" ht="12.8">
       <c r="A29" s="5" t="s">
         <v>81</v>
       </c>
@@ -1190,7 +1196,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="30" ht="12.8">
       <c r="A30" s="5" t="s">
         <v>84</v>
       </c>
@@ -1204,7 +1210,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="31" ht="12.8">
       <c r="A31" s="5" t="s">
         <v>87</v>
       </c>
@@ -1218,7 +1224,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" ht="12.8">
       <c r="A32" s="5" t="s">
         <v>90</v>
       </c>
@@ -1232,7 +1238,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" ht="12.8">
       <c r="A33" s="5" t="s">
         <v>93</v>
       </c>
@@ -1246,7 +1252,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="34" ht="12.8">
       <c r="A34" s="5" t="s">
         <v>96</v>
       </c>
@@ -1260,7 +1266,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="35" ht="12.8">
       <c r="A35" s="5" t="s">
         <v>99</v>
       </c>
@@ -1274,7 +1280,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="36" ht="12.8">
       <c r="A36" s="5" t="s">
         <v>102</v>
       </c>
@@ -1288,7 +1294,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="37" ht="12.8">
       <c r="A37" s="5" t="s">
         <v>105</v>
       </c>
@@ -1302,7 +1308,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="38" ht="12.8">
       <c r="A38" s="5" t="s">
         <v>108</v>
       </c>
@@ -1316,7 +1322,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="39" ht="12.8">
       <c r="A39" s="5" t="s">
         <v>111</v>
       </c>
@@ -1330,7 +1336,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="40" ht="12.8">
       <c r="A40" s="5" t="s">
         <v>114</v>
       </c>
@@ -1344,7 +1350,7 @@
         <v>116</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="41" ht="12.8">
       <c r="A41" s="5" t="s">
         <v>117</v>
       </c>
@@ -1361,12 +1367,12 @@
   </sheetData>
   <autoFilter ref="A3:D4"/>
   <conditionalFormatting sqref="A1:A63578">
-    <cfRule type="duplicateValues" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="2"/>
   </conditionalFormatting>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0" gridLinesSet="1"/>
   <pageMargins left="0.747916666666667" right="0.747916666666667" top="0.984027777777778" bottom="0.984027777777778" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" orientation="portrait" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter>
     <oddHeader/>
     <oddFooter/>
   </headerFooter>

</xml_diff>